<commit_message>
Update C4 viewer (C6-9)
</commit_message>
<xml_diff>
--- a/c6b/downloads/C6B/SkyG-Speed-90B-C6B-11-BOM.xlsx
+++ b/c6b/downloads/C6B/SkyG-Speed-90B-C6B-11-BOM.xlsx
@@ -1103,7 +1103,11 @@
           <t>Class</t>
         </is>
       </c>
-      <c r="J16" s="8" t="inlineStr"/>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>Owner 2026-10-11: XT30 kept (ready-made 4S 650 packs have XT30). Rated 30 A peak; the F50 + Gemfan draw 33-36 A at full power: passes of 10 s or less</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">

</xml_diff>